<commit_message>
Added New Word Upload Feature and Multi Env Deployment Code
</commit_message>
<xml_diff>
--- a/Backend/flashMobGre/src/main/resources/Words.xlsx
+++ b/Backend/flashMobGre/src/main/resources/Words.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="153222"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GRE\"/>
     </mc:Choice>
@@ -17,7 +17,7 @@
   <calcPr calcId="152511"/>
   <fileRecoveryPr repairLoad="1"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2228" uniqueCount="2206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2236" uniqueCount="2214">
   <si>
     <t>Name</t>
   </si>
@@ -7187,11 +7187,36 @@
   <si>
     <t>1. दारिद्र्य</t>
   </si>
+  <si>
+    <t>Resilience</t>
+  </si>
+  <si>
+    <t>लवचिकता / संकटातून सावरण्याची क्षमता</t>
+  </si>
+  <si>
+    <t>The ability to recover quickly from difficulties or challenges.</t>
+  </si>
+  <si>
+    <t>Her resilience helped her stay strong after many failures.</t>
+  </si>
+  <si>
+    <t>Ineffable</t>
+  </si>
+  <si>
+    <t>अवर्णनीय / शब्दांत व्यक्त न करता येणारे</t>
+  </si>
+  <si>
+    <t>Too great, beautiful, or powerful to be described in words.</t>
+  </si>
+  <si>
+    <t>The view from the mountain was ineffable.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -7530,15 +7555,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D557"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D559"/>
   <sheetFormatPr defaultRowHeight="60" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.77734375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="19" style="2" customWidth="1"/>
-    <col min="3" max="3" width="83" style="2" customWidth="1"/>
-    <col min="4" max="4" width="98.33203125" style="2" customWidth="1"/>
-    <col min="5" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="1" customWidth="true" style="2" width="17.77734375" collapsed="true"/>
+    <col min="2" max="2" customWidth="true" style="2" width="19.0" collapsed="true"/>
+    <col min="3" max="3" customWidth="true" style="2" width="83.0" collapsed="true"/>
+    <col min="4" max="4" customWidth="true" style="2" width="98.33203125" collapsed="true"/>
+    <col min="5" max="16384" style="2" width="8.88671875" collapsed="true"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.3">
@@ -15339,6 +15364,34 @@
         <v>2204</v>
       </c>
     </row>
+    <row r="558">
+      <c r="A558" t="s">
+        <v>2206</v>
+      </c>
+      <c r="B558" t="s">
+        <v>2207</v>
+      </c>
+      <c r="C558" t="s">
+        <v>2208</v>
+      </c>
+      <c r="D558" t="s">
+        <v>2209</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="s">
+        <v>2210</v>
+      </c>
+      <c r="B559" t="s">
+        <v>2211</v>
+      </c>
+      <c r="C559" t="s">
+        <v>2212</v>
+      </c>
+      <c r="D559" t="s">
+        <v>2213</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>